<commit_message>
Update admissions dashboard data
</commit_message>
<xml_diff>
--- a/DATA/manual-dashboard-data-2025.xlsx
+++ b/DATA/manual-dashboard-data-2025.xlsx
@@ -10,10 +10,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="8" width="18" customWidth="1"/>
+    <col min="2" max="12" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -57,6 +57,11 @@
           <t>26.06.2025</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>27.06.2025</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -84,11 +89,17 @@
         <v>145</v>
       </c>
       <c r="F3">
-        <v>221</v>
+        <v>170</v>
       </c>
       <c r="G3">
         <v>181</v>
       </c>
+      <c r="H3">
+        <v>120</v>
+      </c>
+      <c r="I3">
+        <v>80</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -116,10 +127,16 @@
         <v>145</v>
       </c>
       <c r="F5">
-        <v>221</v>
+        <v>170</v>
       </c>
       <c r="G5">
         <v>181</v>
+      </c>
+      <c r="H5">
+        <v>120</v>
+      </c>
+      <c r="I5">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -128,10 +145,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I7"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="8" width="18" customWidth="1"/>
+    <col min="2" max="12" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -175,6 +192,11 @@
           <t>26.06.2025</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>27.06.2025</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -270,6 +292,12 @@
       </c>
       <c r="G7">
         <v>181</v>
+      </c>
+      <c r="H7">
+        <v>120</v>
+      </c>
+      <c r="I7">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update admissions data and remove browser cache
</commit_message>
<xml_diff>
--- a/DATA/manual-dashboard-data-2025.xlsx
+++ b/DATA/manual-dashboard-data-2025.xlsx
@@ -13,7 +13,7 @@
   <dimension ref="A1:I5"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="12" width="18" customWidth="1"/>
+    <col min="2" max="32" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -148,7 +148,7 @@
   <dimension ref="A1:I7"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
-    <col min="2" max="12" width="18" customWidth="1"/>
+    <col min="2" max="32" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add unused specialties dashboard block
</commit_message>
<xml_diff>
--- a/DATA/manual-dashboard-data-2025.xlsx
+++ b/DATA/manual-dashboard-data-2025.xlsx
@@ -10,7 +10,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:P5"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="32" width="18" customWidth="1"/>
@@ -29,37 +29,72 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>21.06.2025</t>
+          <t>22.06.2025</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>22.06.2025</t>
+          <t>23.06.2025</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>23.06.2025</t>
+          <t>24.06.2025</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>24.06.2025</t>
+          <t>25.06.2025</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>25.06.2025</t>
+          <t>26.06.2025</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>26.06.2025</t>
+          <t>27.06.2025</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>27.06.2025</t>
+          <t>29.06.2025</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>30.06.2025</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>01.07.2025</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>02.07.2025</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>03.07.2025</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>04.07.2025</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>06.07.2025</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>07.07.2025</t>
         </is>
       </c>
     </row>
@@ -77,28 +112,49 @@
         </is>
       </c>
       <c r="B3">
-        <v>196</v>
+        <v>35</v>
       </c>
       <c r="C3">
-        <v>67</v>
+        <v>42</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="E3">
-        <v>145</v>
+        <v>72</v>
       </c>
       <c r="F3">
-        <v>170</v>
+        <v>21</v>
       </c>
       <c r="G3">
-        <v>181</v>
+        <v>26</v>
       </c>
       <c r="H3">
+        <v>8</v>
+      </c>
+      <c r="I3">
+        <v>96</v>
+      </c>
+      <c r="J3">
+        <v>139</v>
+      </c>
+      <c r="K3">
+        <v>112</v>
+      </c>
+      <c r="L3">
         <v>120</v>
       </c>
-      <c r="I3">
-        <v>80</v>
+      <c r="M3">
+        <v>256</v>
+      </c>
+      <c r="N3">
+        <v>37</v>
+      </c>
+      <c r="O3">
+        <v>142</v>
+      </c>
+      <c r="P3">
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -115,28 +171,49 @@
         </is>
       </c>
       <c r="B5">
-        <v>196</v>
+        <v>35</v>
       </c>
       <c r="C5">
-        <v>67</v>
+        <v>42</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="E5">
-        <v>145</v>
+        <v>72</v>
       </c>
       <c r="F5">
-        <v>170</v>
+        <v>21</v>
       </c>
       <c r="G5">
-        <v>181</v>
+        <v>26</v>
       </c>
       <c r="H5">
+        <v>8</v>
+      </c>
+      <c r="I5">
+        <v>96</v>
+      </c>
+      <c r="J5">
+        <v>139</v>
+      </c>
+      <c r="K5">
+        <v>112</v>
+      </c>
+      <c r="L5">
         <v>120</v>
       </c>
-      <c r="I5">
-        <v>80</v>
+      <c r="M5">
+        <v>256</v>
+      </c>
+      <c r="N5">
+        <v>37</v>
+      </c>
+      <c r="O5">
+        <v>142</v>
+      </c>
+      <c r="P5">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -145,7 +222,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:S7"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="32" width="18" customWidth="1"/>
@@ -197,6 +274,56 @@
           <t>27.06.2025</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>28.06.2025</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>29.06.2025</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>30.06.2025</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>01.07.2025</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>02.07.2025</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>03.07.2025</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>04.07.2025</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>05.07.2025</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>06.07.2025</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>07.07.2025</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -205,22 +332,58 @@
         </is>
       </c>
       <c r="B2">
-        <v>175</v>
+        <v>138</v>
       </c>
       <c r="C2">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="E2">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="F2">
-        <v>192</v>
+        <v>150</v>
       </c>
       <c r="G2">
-        <v>159</v>
+        <v>119</v>
+      </c>
+      <c r="H2">
+        <v>108</v>
+      </c>
+      <c r="I2">
+        <v>97</v>
+      </c>
+      <c r="J2">
+        <v>15</v>
+      </c>
+      <c r="K2">
+        <v>232</v>
+      </c>
+      <c r="L2">
+        <v>254</v>
+      </c>
+      <c r="M2">
+        <v>233</v>
+      </c>
+      <c r="N2">
+        <v>232</v>
+      </c>
+      <c r="O2">
+        <v>156</v>
+      </c>
+      <c r="P2">
+        <v>123</v>
+      </c>
+      <c r="Q2">
+        <v>9</v>
+      </c>
+      <c r="R2">
+        <v>178</v>
+      </c>
+      <c r="S2">
+        <v>37</v>
       </c>
     </row>
     <row r="3">
@@ -230,22 +393,58 @@
         </is>
       </c>
       <c r="B3">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="C3">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F3">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>22</v>
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>5</v>
+      </c>
+      <c r="I3">
+        <v>3</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>10</v>
+      </c>
+      <c r="L3">
+        <v>9</v>
+      </c>
+      <c r="M3">
+        <v>6</v>
+      </c>
+      <c r="N3">
+        <v>9</v>
+      </c>
+      <c r="O3">
+        <v>4</v>
+      </c>
+      <c r="P3">
+        <v>5</v>
+      </c>
+      <c r="Q3">
+        <v>3</v>
+      </c>
+      <c r="R3">
+        <v>6</v>
+      </c>
+      <c r="S3">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -254,6 +453,60 @@
           <t>Целевая квота</t>
         </is>
       </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -261,6 +514,60 @@
           <t>Отдельная квота</t>
         </is>
       </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -268,6 +575,60 @@
           <t>Особая квота</t>
         </is>
       </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <v>0</v>
+      </c>
+      <c r="R6">
+        <v>0</v>
+      </c>
+      <c r="S6">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -276,28 +637,58 @@
         </is>
       </c>
       <c r="B7">
-        <v>196</v>
+        <v>142</v>
       </c>
       <c r="C7">
-        <v>67</v>
+        <v>12</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="E7">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="F7">
-        <v>221</v>
+        <v>153</v>
       </c>
       <c r="G7">
-        <v>181</v>
+        <v>121</v>
       </c>
       <c r="H7">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="I7">
-        <v>80</v>
+        <v>100</v>
+      </c>
+      <c r="J7">
+        <v>17</v>
+      </c>
+      <c r="K7">
+        <v>242</v>
+      </c>
+      <c r="L7">
+        <v>263</v>
+      </c>
+      <c r="M7">
+        <v>239</v>
+      </c>
+      <c r="N7">
+        <v>241</v>
+      </c>
+      <c r="O7">
+        <v>160</v>
+      </c>
+      <c r="P7">
+        <v>128</v>
+      </c>
+      <c r="Q7">
+        <v>12</v>
+      </c>
+      <c r="R7">
+        <v>184</v>
+      </c>
+      <c r="S7">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update dashboard manual data and KCP summary
</commit_message>
<xml_diff>
--- a/DATA/manual-dashboard-data-2025.xlsx
+++ b/DATA/manual-dashboard-data-2025.xlsx
@@ -112,49 +112,49 @@
         </is>
       </c>
       <c r="B3">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="C3">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D3">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="E3">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="F3">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G3">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="H3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I3">
-        <v>96</v>
+        <v>137</v>
       </c>
       <c r="J3">
-        <v>139</v>
+        <v>91</v>
       </c>
       <c r="K3">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="L3">
-        <v>120</v>
+        <v>74</v>
       </c>
       <c r="M3">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="N3">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="O3">
-        <v>142</v>
+        <v>118</v>
       </c>
       <c r="P3">
-        <v>15</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
@@ -171,49 +171,49 @@
         </is>
       </c>
       <c r="B5">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="C5">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D5">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="E5">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="F5">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G5">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="H5">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I5">
-        <v>96</v>
+        <v>137</v>
       </c>
       <c r="J5">
-        <v>139</v>
+        <v>91</v>
       </c>
       <c r="K5">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="L5">
-        <v>120</v>
+        <v>74</v>
       </c>
       <c r="M5">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="N5">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="O5">
-        <v>142</v>
+        <v>118</v>
       </c>
       <c r="P5">
-        <v>15</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -332,58 +332,58 @@
         </is>
       </c>
       <c r="B2">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C2">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D2">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E2">
-        <v>133</v>
+        <v>75</v>
       </c>
       <c r="F2">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="G2">
-        <v>119</v>
+        <v>106</v>
       </c>
       <c r="H2">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="I2">
-        <v>97</v>
+        <v>64</v>
       </c>
       <c r="J2">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="K2">
-        <v>232</v>
+        <v>194</v>
       </c>
       <c r="L2">
-        <v>254</v>
+        <v>174</v>
       </c>
       <c r="M2">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="N2">
-        <v>232</v>
+        <v>78</v>
       </c>
       <c r="O2">
-        <v>156</v>
+        <v>270</v>
       </c>
       <c r="P2">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="Q2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="R2">
-        <v>178</v>
+        <v>226</v>
       </c>
       <c r="S2">
-        <v>37</v>
+        <v>221</v>
       </c>
     </row>
     <row r="3">
@@ -393,58 +393,58 @@
         </is>
       </c>
       <c r="B3">
+        <v>6</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>7</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
         <v>4</v>
       </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-      <c r="E3">
+      <c r="G3">
         <v>3</v>
       </c>
-      <c r="F3">
+      <c r="H3">
+        <v>9</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>5</v>
+      </c>
+      <c r="L3">
+        <v>7</v>
+      </c>
+      <c r="M3">
+        <v>4</v>
+      </c>
+      <c r="N3">
         <v>3</v>
       </c>
-      <c r="G3">
-        <v>2</v>
-      </c>
-      <c r="H3">
-        <v>5</v>
-      </c>
-      <c r="I3">
-        <v>3</v>
-      </c>
-      <c r="J3">
-        <v>2</v>
-      </c>
-      <c r="K3">
+      <c r="O3">
         <v>10</v>
       </c>
-      <c r="L3">
-        <v>9</v>
-      </c>
-      <c r="M3">
-        <v>6</v>
-      </c>
-      <c r="N3">
-        <v>9</v>
-      </c>
-      <c r="O3">
-        <v>4</v>
-      </c>
       <c r="P3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="R3">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="S3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -460,19 +460,19 @@
         <v>0</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G4">
         <v>0</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -481,19 +481,19 @@
         <v>0</v>
       </c>
       <c r="K4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N4">
         <v>0</v>
       </c>
       <c r="O4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P4">
         <v>0</v>
@@ -502,7 +502,7 @@
         <v>0</v>
       </c>
       <c r="R4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S4">
         <v>0</v>
@@ -518,7 +518,7 @@
         <v>0</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -527,7 +527,7 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -536,7 +536,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5">
         <v>0</v>
@@ -545,7 +545,7 @@
         <v>0</v>
       </c>
       <c r="L5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M5">
         <v>0</v>
@@ -554,7 +554,7 @@
         <v>0</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P5">
         <v>0</v>
@@ -563,10 +563,10 @@
         <v>0</v>
       </c>
       <c r="R5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S5">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -576,25 +576,25 @@
         </is>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E6">
         <v>0</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I6">
         <v>0</v>
@@ -603,31 +603,31 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M6">
         <v>0</v>
       </c>
       <c r="N6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O6">
         <v>0</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
       <c r="R6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S6">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -637,58 +637,58 @@
         </is>
       </c>
       <c r="B7">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="C7">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D7">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="E7">
-        <v>136</v>
+        <v>77</v>
       </c>
       <c r="F7">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="G7">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="H7">
-        <v>113</v>
+        <v>143</v>
       </c>
       <c r="I7">
-        <v>100</v>
+        <v>66</v>
       </c>
       <c r="J7">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="K7">
+        <v>201</v>
+      </c>
+      <c r="L7">
+        <v>184</v>
+      </c>
+      <c r="M7">
+        <v>247</v>
+      </c>
+      <c r="N7">
+        <v>82</v>
+      </c>
+      <c r="O7">
+        <v>282</v>
+      </c>
+      <c r="P7">
+        <v>130</v>
+      </c>
+      <c r="Q7">
+        <v>9</v>
+      </c>
+      <c r="R7">
         <v>242</v>
       </c>
-      <c r="L7">
-        <v>263</v>
-      </c>
-      <c r="M7">
-        <v>239</v>
-      </c>
-      <c r="N7">
-        <v>241</v>
-      </c>
-      <c r="O7">
-        <v>160</v>
-      </c>
-      <c r="P7">
-        <v>128</v>
-      </c>
-      <c r="Q7">
-        <v>12</v>
-      </c>
-      <c r="R7">
-        <v>184</v>
-      </c>
       <c r="S7">
-        <v>38</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update previous year applicants series
</commit_message>
<xml_diff>
--- a/DATA/manual-dashboard-data-2025.xlsx
+++ b/DATA/manual-dashboard-data-2025.xlsx
@@ -10,7 +10,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:AA5"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="32" width="18" customWidth="1"/>
@@ -24,77 +24,132 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>19.06.2025</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>20.06.2025</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>22.06.2025</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>23.06.2025</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>24.06.2025</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>25.06.2025</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>26.06.2025</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>27.06.2025</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>29.06.2025</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>30.06.2025</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>01.07.2025</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>02.07.2025</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>03.07.2025</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>04.07.2025</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>06.07.2025</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>07.07.2025</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>08.07.2025</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>09.07.2025</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>10.07.2025</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>11.07.2025</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>13.07.2025</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>14.07.2025</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>15.07.2025</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>16.07.2025</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>17.07.2025</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>18.07.2025</t>
         </is>
       </c>
     </row>
@@ -112,49 +167,82 @@
         </is>
       </c>
       <c r="B3">
-        <v>49</v>
+        <v>196</v>
       </c>
       <c r="C3">
-        <v>34</v>
+        <v>67</v>
       </c>
       <c r="D3">
-        <v>58</v>
+        <v>145</v>
       </c>
       <c r="E3">
-        <v>64</v>
+        <v>221</v>
       </c>
       <c r="F3">
-        <v>19</v>
+        <v>181</v>
       </c>
       <c r="G3">
-        <v>51</v>
+        <v>189</v>
       </c>
       <c r="H3">
-        <v>12</v>
+        <v>189</v>
       </c>
       <c r="I3">
-        <v>137</v>
+        <v>109</v>
       </c>
       <c r="J3">
-        <v>91</v>
+        <v>308</v>
       </c>
       <c r="K3">
-        <v>129</v>
+        <v>296</v>
       </c>
       <c r="L3">
-        <v>74</v>
+        <v>206</v>
       </c>
       <c r="M3">
-        <v>252</v>
+        <v>286</v>
       </c>
       <c r="N3">
-        <v>43</v>
+        <v>235</v>
       </c>
       <c r="O3">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="P3">
-        <v>27</v>
+        <v>253</v>
+      </c>
+      <c r="Q3">
+        <v>244</v>
+      </c>
+      <c r="R3">
+        <v>217</v>
+      </c>
+      <c r="S3">
+        <v>211</v>
+      </c>
+      <c r="T3">
+        <v>241</v>
+      </c>
+      <c r="U3">
+        <v>101</v>
+      </c>
+      <c r="V3">
+        <v>284</v>
+      </c>
+      <c r="W3">
+        <v>206</v>
+      </c>
+      <c r="X3">
+        <v>240</v>
+      </c>
+      <c r="Y3">
+        <v>258</v>
+      </c>
+      <c r="Z3">
+        <v>153</v>
+      </c>
+      <c r="AA3">
+        <v>135</v>
       </c>
     </row>
     <row r="4">
@@ -171,49 +259,82 @@
         </is>
       </c>
       <c r="B5">
-        <v>49</v>
+        <v>196</v>
       </c>
       <c r="C5">
-        <v>34</v>
+        <v>67</v>
       </c>
       <c r="D5">
-        <v>58</v>
+        <v>145</v>
       </c>
       <c r="E5">
-        <v>64</v>
+        <v>221</v>
       </c>
       <c r="F5">
-        <v>19</v>
+        <v>181</v>
       </c>
       <c r="G5">
-        <v>51</v>
+        <v>189</v>
       </c>
       <c r="H5">
-        <v>12</v>
+        <v>189</v>
       </c>
       <c r="I5">
-        <v>137</v>
+        <v>109</v>
       </c>
       <c r="J5">
-        <v>91</v>
+        <v>308</v>
       </c>
       <c r="K5">
-        <v>129</v>
+        <v>296</v>
       </c>
       <c r="L5">
-        <v>74</v>
+        <v>206</v>
       </c>
       <c r="M5">
-        <v>252</v>
+        <v>286</v>
       </c>
       <c r="N5">
-        <v>43</v>
+        <v>235</v>
       </c>
       <c r="O5">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="P5">
-        <v>27</v>
+        <v>253</v>
+      </c>
+      <c r="Q5">
+        <v>244</v>
+      </c>
+      <c r="R5">
+        <v>217</v>
+      </c>
+      <c r="S5">
+        <v>211</v>
+      </c>
+      <c r="T5">
+        <v>241</v>
+      </c>
+      <c r="U5">
+        <v>101</v>
+      </c>
+      <c r="V5">
+        <v>284</v>
+      </c>
+      <c r="W5">
+        <v>206</v>
+      </c>
+      <c r="X5">
+        <v>240</v>
+      </c>
+      <c r="Y5">
+        <v>258</v>
+      </c>
+      <c r="Z5">
+        <v>153</v>
+      </c>
+      <c r="AA5">
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update admission dashboard data for August
</commit_message>
<xml_diff>
--- a/DATA/manual-dashboard-data-2025.xlsx
+++ b/DATA/manual-dashboard-data-2025.xlsx
@@ -10,7 +10,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA5"/>
+  <dimension ref="A1:AR5"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="32" width="18" customWidth="1"/>
@@ -152,6 +152,91 @@
           <t>18.07.2025</t>
         </is>
       </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>20.07.2025</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>22.07.2025</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>23.07.2025</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>24.07.2025</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>25.07.2025</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>27.07.2025</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>28.07.2025</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>29.07.2025</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>30.07.2025</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>31.07.2025</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>01.08.2025</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>03.08.2025</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>04.08.2025</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>05.08.2025</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>06.08.2025</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>07.08.2025</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>10.08.2025</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -244,6 +329,57 @@
       <c r="AA3">
         <v>135</v>
       </c>
+      <c r="AB3">
+        <v>74</v>
+      </c>
+      <c r="AC3">
+        <v>84</v>
+      </c>
+      <c r="AD3">
+        <v>26</v>
+      </c>
+      <c r="AE3">
+        <v>22</v>
+      </c>
+      <c r="AF3">
+        <v>8</v>
+      </c>
+      <c r="AG3">
+        <v>34</v>
+      </c>
+      <c r="AH3">
+        <v>0</v>
+      </c>
+      <c r="AI3">
+        <v>86</v>
+      </c>
+      <c r="AJ3">
+        <v>52</v>
+      </c>
+      <c r="AK3">
+        <v>21</v>
+      </c>
+      <c r="AL3">
+        <v>13</v>
+      </c>
+      <c r="AM3">
+        <v>58</v>
+      </c>
+      <c r="AN3">
+        <v>101</v>
+      </c>
+      <c r="AO3">
+        <v>72</v>
+      </c>
+      <c r="AP3">
+        <v>87</v>
+      </c>
+      <c r="AQ3">
+        <v>86</v>
+      </c>
+      <c r="AR3">
+        <v>116</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -335,6 +471,57 @@
       </c>
       <c r="AA5">
         <v>135</v>
+      </c>
+      <c r="AB5">
+        <v>74</v>
+      </c>
+      <c r="AC5">
+        <v>84</v>
+      </c>
+      <c r="AD5">
+        <v>26</v>
+      </c>
+      <c r="AE5">
+        <v>22</v>
+      </c>
+      <c r="AF5">
+        <v>8</v>
+      </c>
+      <c r="AG5">
+        <v>34</v>
+      </c>
+      <c r="AH5">
+        <v>0</v>
+      </c>
+      <c r="AI5">
+        <v>86</v>
+      </c>
+      <c r="AJ5">
+        <v>52</v>
+      </c>
+      <c r="AK5">
+        <v>21</v>
+      </c>
+      <c r="AL5">
+        <v>13</v>
+      </c>
+      <c r="AM5">
+        <v>58</v>
+      </c>
+      <c r="AN5">
+        <v>101</v>
+      </c>
+      <c r="AO5">
+        <v>72</v>
+      </c>
+      <c r="AP5">
+        <v>87</v>
+      </c>
+      <c r="AQ5">
+        <v>86</v>
+      </c>
+      <c r="AR5">
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>